<commit_message>
Update daily log for August 19, 2026
</commit_message>
<xml_diff>
--- a/daily-log-1.xlsx
+++ b/daily-log-1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/B0AA7295676BA96C/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{370DD9F5-B5DD-4EFC-93C9-87386ADFAB99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="15" documentId="8_{370DD9F5-B5DD-4EFC-93C9-87386ADFAB99}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{97535FCB-FD16-443D-B1AA-649F6F8148BF}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="61">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -212,6 +212,12 @@
   </si>
   <si>
     <t>Attended 4 classes, completed 3 hours of study and 1 hour of coding. Also completed 30 minutes of fitness and other activities. Overall, it was a productive day</t>
+  </si>
+  <si>
+    <t>Studied for 7 hours and completed 2 hours of coding. Also completed 30 minutes of fitness and other activities. No classes were attended today. Overall, it was a productive day</t>
+  </si>
+  <si>
+    <t>Low</t>
   </si>
 </sst>
 </file>
@@ -492,6 +498,10 @@
 </styleSheet>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -1082,27 +1092,51 @@
         <v>58</v>
       </c>
     </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="A8" s="13"/>
-      <c r="B8" s="14"/>
-      <c r="C8" s="14"/>
-      <c r="D8" s="14"/>
-      <c r="E8" s="14"/>
-      <c r="F8" s="14"/>
-      <c r="G8" s="14"/>
-      <c r="H8" s="14"/>
-      <c r="I8" s="15" t="str">
+    <row r="8" spans="1:14" ht="105" x14ac:dyDescent="0.25">
+      <c r="A8" s="13">
+        <v>46253</v>
+      </c>
+      <c r="B8" s="14">
+        <v>480</v>
+      </c>
+      <c r="C8" s="14">
+        <v>30</v>
+      </c>
+      <c r="D8" s="14">
+        <v>420</v>
+      </c>
+      <c r="E8" s="14">
+        <v>120</v>
+      </c>
+      <c r="F8" s="14">
+        <v>0</v>
+      </c>
+      <c r="G8" s="14">
+        <v>0</v>
+      </c>
+      <c r="H8" s="14">
+        <v>30</v>
+      </c>
+      <c r="I8" s="15">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J8" s="15" t="str">
+        <v>1080</v>
+      </c>
+      <c r="J8" s="15">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K8" s="16"/>
-      <c r="L8" s="16"/>
-      <c r="M8" s="16"/>
-      <c r="N8" s="17"/>
+        <v>360</v>
+      </c>
+      <c r="K8" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="L8" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="M8" s="16" t="s">
+        <v>60</v>
+      </c>
+      <c r="N8" s="17" t="s">
+        <v>59</v>
+      </c>
     </row>
     <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" s="13"/>

</xml_diff>